<commit_message>
fix to fig 2
</commit_message>
<xml_diff>
--- a/display_items/supplement.xlsx
+++ b/display_items/supplement.xlsx
@@ -48526,13 +48526,13 @@
         <v>7</v>
       </c>
       <c r="D2" t="n">
-        <v>0.00393253851620032</v>
+        <v>0.0248987711059041</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.00377509534336889</v>
+        <v>0.0158527009148992</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0116401723757695</v>
+        <v>0.0339448412969091</v>
       </c>
     </row>
     <row r="3">
@@ -48546,13 +48546,13 @@
         <v>7</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0156557772023518</v>
+        <v>0.0402574241050405</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0086850396411385</v>
+        <v>0.0332866865438272</v>
       </c>
       <c r="F3" t="n">
-        <v>0.022626514763565</v>
+        <v>0.0472281616662538</v>
       </c>
     </row>
     <row r="4">
@@ -48566,13 +48566,13 @@
         <v>7</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0818406538327087</v>
+        <v>0.106442300735397</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0701660597246842</v>
+        <v>0.0947677066273729</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0935152479407332</v>
+        <v>0.118116894843422</v>
       </c>
     </row>
     <row r="5">
@@ -48586,13 +48586,13 @@
         <v>7</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1380243157667</v>
+        <v>0.162625962669389</v>
       </c>
       <c r="E5" t="n">
-        <v>0.121997954446821</v>
+        <v>0.14659960134951</v>
       </c>
       <c r="F5" t="n">
-        <v>0.15405067708658</v>
+        <v>0.178652323989268</v>
       </c>
     </row>
     <row r="6">
@@ -48606,13 +48606,13 @@
         <v>7</v>
       </c>
       <c r="D6" t="n">
-        <v>0.180095680744755</v>
+        <v>0.204697327647444</v>
       </c>
       <c r="E6" t="n">
-        <v>0.15882786442698</v>
+        <v>0.183429511329669</v>
       </c>
       <c r="F6" t="n">
-        <v>0.201363497062531</v>
+        <v>0.225965143965219</v>
       </c>
     </row>
     <row r="7">
@@ -48626,13 +48626,13 @@
         <v>11</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>0.0987896921898958</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>0.087616267398702</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>0.10996311698109</v>
       </c>
     </row>
     <row r="8">
@@ -48646,13 +48646,13 @@
         <v>11</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0476942338519166</v>
+        <v>0.178422989670676</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0170246430059675</v>
+        <v>0.145450930830471</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0783638246978656</v>
+        <v>0.21139504851088</v>
       </c>
     </row>
     <row r="9">
@@ -48666,13 +48666,13 @@
         <v>11</v>
       </c>
       <c r="D9" t="n">
-        <v>0.19139679147705</v>
+        <v>0.324508191673136</v>
       </c>
       <c r="E9" t="n">
-        <v>0.138136061553059</v>
+        <v>0.271247461749145</v>
       </c>
       <c r="F9" t="n">
-        <v>0.244657521401041</v>
+        <v>0.377768921597127</v>
       </c>
     </row>
     <row r="10">
@@ -48686,13 +48686,13 @@
         <v>11</v>
       </c>
       <c r="D10" t="n">
-        <v>0.285730912786005</v>
+        <v>0.418842312982091</v>
       </c>
       <c r="E10" t="n">
-        <v>0.25484239142892</v>
+        <v>0.387953791625006</v>
       </c>
       <c r="F10" t="n">
-        <v>0.31661943414309</v>
+        <v>0.449730834339176</v>
       </c>
     </row>
     <row r="11">
@@ -48706,13 +48706,13 @@
         <v>11</v>
       </c>
       <c r="D11" t="n">
-        <v>0.359714607569073</v>
+        <v>0.492826007765158</v>
       </c>
       <c r="E11" t="n">
-        <v>0.304842175954889</v>
+        <v>0.437953576150975</v>
       </c>
       <c r="F11" t="n">
-        <v>0.414587039183256</v>
+        <v>0.547698439379342</v>
       </c>
     </row>
   </sheetData>

</xml_diff>